<commit_message>
chore: rebuild assets, update Etsy stats, add tasks archive
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etsy_daily_stats.xlsx
+++ b/etsy_daily_stats.xlsx
@@ -91,7 +91,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -132,6 +132,9 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,7 +388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="5" min="1" max="1"/>
@@ -464,42 +467,42 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="6">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="8" t="n">
+      <c r="C2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="H2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Baseline (seeded manually)</t>
         </is>
@@ -542,6 +545,44 @@
         <v>0</v>
       </c>
       <c r="L3" s="11" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="14" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
chore: update etsy daily stats spreadsheet
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etsy_daily_stats.xlsx
+++ b/etsy_daily_stats.xlsx
@@ -388,7 +388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="5" min="1" max="1"/>
@@ -584,6 +584,44 @@
       </c>
       <c r="L4" s="14" t="n"/>
     </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="14" t="n"/>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>